<commit_message>
Added specs for the tenant registration and login
</commit_message>
<xml_diff>
--- a/booklets/user-stories/user-stories.xlsx
+++ b/booklets/user-stories/user-stories.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1898,6 +1898,335 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>US-31</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Tenant admin</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>to register my tenant with its name, my email and a password</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>my team gets its own private workspace</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Puccetti</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Password &gt;= 10 characters, stored hashed with BCrypt; email unique (case-insensitive)</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>US-32</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>to log in and log out</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>only my team can see our data</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Puccetti</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Server session in an HttpOnly, SameSite=Lax cookie; CSRF token on every state-changing request; generic "invalid email or password" message; every `/api` endpoint except register and login returns 401 without a session</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>US-33</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Tenant admin</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>the imports, maps and plans of my tenant to be invisible to any other tenant</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>our confidential revenue data stays private (NDA)</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Puccetti</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Enforced by one backend guard on all `/api/imports/{id}/**` and `/api/plans/{planId}/**` routes; another tenant's id returns 404, not 403; covered by an automated isolation test</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>US-34</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Tenant admin</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>to register the enterprises of my tenant (name, column header in our ERP export, color and optionally VAT number and headquarters address), at registration or later</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>I enter them once instead of at every import</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>S12, S13</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Puccetti</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Optional at registration; name and ERP column unique per tenant (case-insensitive); headquarters geocoded with the same cache and rate limit as delivery points</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>US-35</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Analyst</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>the import wizard to match the file columns to my registered enterprises and pre-fill their names, colors and addresses</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>importing a new yearly file takes fewer steps</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Puccetti</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Case- and accent-insensitive match on the ERP column, then on the name; numeric columns that match nothing are still suggested as new enterprises</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>US-36</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Analyst</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>to change the enterprise data (including the headquarters address) for a single import in the wizard</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>I can try alternatives and see how they change the results</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Puccetti</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Values copied into the import (snapshot); the profile changes only if "Also save to profile" is ticked; editing the profile never changes existing imports</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>US-37</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Tenant admin</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>a profile page to change the tenant name, my password and the enterprises</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>our information stays up to date</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Puccetti</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Password change requires the current password; deleting an enterprise does not change existing imports</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1909,7 +2238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2116,6 +2445,40 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Register / Log in</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>mockups/S12-*.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Tenant profile</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>mockups/S13-*.png</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(booklets): add authentication design and API contract section
Add AUTHENTICATION.md with the scope, the security decisions for
registration, login and profile (one account per tenant, Argon2id,
server session, SPA CSRF, lockout) and the implementation steps.
Add endpoints 19-25 to the API contract and the matching TypeScript
types. Align US-31, US-37, PUC-8 and D-09 with one account per tenant.

Refs: PUC-8, US-31, US-32, US-37
</commit_message>
<xml_diff>
--- a/booklets/user-stories/user-stories.xlsx
+++ b/booklets/user-stories/user-stories.xlsx
@@ -1936,7 +1936,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Password &gt;= 10 characters, stored hashed with BCrypt; email unique (case-insensitive)</t>
+          <t>One account per tenant; password 8-64 characters (minimum configurable), no composition rules, stored hashed with Argon2id (OWASP ASVS 5.0); email unique (case-insensitive)</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>a profile page to change the tenant name, my password and the enterprises</t>
+          <t>a profile page to change the tenant name, the password and the enterprises</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Password change requires the current password; deleting an enterprise does not change existing imports</t>
+          <t>Password change requires the current password and logs out the other sessions; deleting an enterprise does not change existing imports</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs(booklets): replace enterprise registry with tenant starting base
Drop the enterprise registry stories (registration, profile, wizard
pre-fill) and renumber the profile story to US-34. Add US-35: one
starting base per tenant, set by address in the planner form and used
as the plan base. Add endpoints 26-27 and their types, decision D-10
and task PUC-10; align US-21 and the optimization defaults.

Refs: PUC-10, US-21, US-34, US-35
</commit_message>
<xml_diff>
--- a/booklets/user-stories/user-stories.xlsx
+++ b/booklets/user-stories/user-stories.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1441,7 +1441,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>to set the visit parameters (visit duration, working hours, starting point, maximum distance)</t>
+          <t>to set the visit parameters (visit duration, working hours, maximum distance)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Defaults: visit 210 min, workday 480 min, base Rome centre, max 80 km; invalid values rejected with a clear message</t>
+          <t>Defaults: visit 210 min, workday 480 min, max 80 km; every day starts and ends at the tenant starting base (US-35); invalid values rejected with a clear message</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -2052,12 +2052,12 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>to register the enterprises of my tenant (name, column header in our ERP export, color and optionally VAT number and headquarters address), at registration or later</t>
+          <t>a profile page to change the tenant name and the password</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>I enter them once instead of at every import</t>
+          <t>our information stays up to date</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>S12, S13</t>
+          <t>S13</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Optional at registration; name and ERP column unique per tenant (case-insensitive); headquarters geocoded with the same cache and rate limit as delivery points</t>
+          <t>Password change requires the current password and logs out the other sessions</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2099,12 +2099,12 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>the import wizard to match the file columns to my registered enterprises and pre-fill their names, colors and addresses</t>
+          <t>to set the starting base of my tenant once by typing its address in the planner</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>importing a new yearly file takes fewer steps</t>
+          <t>every plan starts from our real base without entering it again</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>S7</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -2124,104 +2124,10 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Case- and accent-insensitive match on the ERP column, then on the name; numeric columns that match nothing are still suggested as new enterprises</t>
+          <t>One base per tenant, stored in the database; address + city geocoded with the Nominatim cache and rate limit; address not found -&gt; clear message and the saved base unchanged; until a base is set the planner uses the configured default (Rome centre)</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>US-36</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>Analyst</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>to change the enterprise data (including the headquarters address) for a single import in the wizard</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>I can try alternatives and see how they change the results</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>Should</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>S4</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>Puccetti</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>Values copied into the import (snapshot); the profile changes only if "Also save to profile" is ticked; editing the profile never changes existing imports</t>
-        </is>
-      </c>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>US-37</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Tenant admin</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>a profile page to change the tenant name, the password and the enterprises</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>our information stays up to date</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Should</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>S13</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>Puccetti</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>Password change requires the current password and logs out the other sessions; deleting an enterprise does not change existing imports</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr">
         <is>
           <t>TODO</t>
         </is>

</xml_diff>

<commit_message>
docs(booklets): add user story US-36 for dark mode
Add US-36 (switch between light and dark mode, following the operating
system until the user chooses) to input.txt, USER_STORIES.md and the
stories spreadsheet, and task PUC-11 to the task board.

Refs: PUC-11, US-36
</commit_message>
<xml_diff>
--- a/booklets/user-stories/user-stories.xlsx
+++ b/booklets/user-stories/user-stories.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2128,6 +2128,53 @@
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>US-36</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>to switch the interface between light and dark mode</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>I can work comfortably in any light</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>All (header)</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Puccetti</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Follows the operating system setting until the user chooses; the choice is remembered in the browser; no flash of the wrong theme on load; toggle reachable by keyboard with its state announced to screen readers; text contrast WCAG AA in both themes; also available before login</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
         <is>
           <t>TODO</t>
         </is>

</xml_diff>

<commit_message>
docs(booklets): update docs and story status for the import wizard
Set US-01..US-07 and US-36 to REVIEW and US-31..US-34 (merged login
work) to DONE in USER_STORIES.md and the spreadsheet. Student_doc.md:
add story 36, the dark theme of the frontend and how uploaded files are
handled (temporary file deleted after reading, size and row limits).
TASKS.md: PUC-1 skipped, teammates import the synthetic sample with the
wizard; MAR-3 and RIV-2 now depend on PUC-3. API_CONTRACT.md: skipped
rows, upload limits and the import request checks as implemented.

Refs: PUC-5, PUC-7, PUC-11
</commit_message>
<xml_diff>
--- a/booklets/user-stories/user-stories.xlsx
+++ b/booklets/user-stories/user-stories.xlsx
@@ -531,7 +531,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>REVIEW</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>REVIEW</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>REVIEW</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>REVIEW</t>
         </is>
       </c>
     </row>
@@ -719,7 +719,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>REVIEW</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>REVIEW</t>
         </is>
       </c>
     </row>
@@ -813,7 +813,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>REVIEW</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
     </row>
@@ -1988,7 +1988,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2035,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
     </row>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DONE</t>
         </is>
       </c>
     </row>
@@ -2176,7 +2176,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>REVIEW</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(booklets): add US-37 and the remember-me design
Add user story US-37 (stay logged in on my own device) to input.txt,
USER_STORIES.md, the spreadsheet and Student_doc.md, and task PUC-12.
AUTHENTICATION.md: decision A13 for persistent remember-me tokens.
API_CONTRACT.md and Student_doc.md: the optional remember-me login
parameter, logout and password change forgetting devices, and the
persistent_logins table.

Refs: PUC-12, US-37
</commit_message>
<xml_diff>
--- a/booklets/user-stories/user-stories.xlsx
+++ b/booklets/user-stories/user-stories.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2175,6 +2175,53 @@
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>US-37</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>to stay logged in on my own device</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>I do not have to type my credentials every day</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Puccetti</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Opt-in checkbox at login, off by default; 14 days (configurable); HttpOnly, SameSite=Lax, Secure over HTTPS cookie; random token stored server-side and replaced at every use, reuse of an old token logs out every remembered device; logout forgets this device only, password change forgets every device; the password is never stored by the application</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
         <is>
           <t>REVIEW</t>
         </is>

</xml_diff>

<commit_message>
feat(engine): implement deterministic visit planning
Group eligible targets, fill working days and improve routes with bounded
local search. Compute coverage, travel and capacity KPIs. Support more
than three daily visits within the time budget and document the agreed
revenue rules.

Add targeted planner tests and update task status, story statuses and the
development log.

Refs: MAR-2, US-22, US-23, US-25
</commit_message>
<xml_diff>
--- a/booklets/user-stories/user-stories.xlsx
+++ b/booklets/user-stories/user-stories.xlsx
@@ -1518,7 +1518,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DOING</t>
         </is>
       </c>
     </row>
@@ -1565,7 +1565,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DOING</t>
         </is>
       </c>
     </row>
@@ -1659,7 +1659,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>DOING</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(booklets): record RIV-4 status and devlog
Adds the RIV-4 section on top of the task status log (RIV-4 in review,
MAR-5 merged with PR #7), sets US-28, US-29 and US-30 to REVIEW in the
user stories and in the spreadsheet, and adds the devlog of the agent
plan page and Excel export.

Refs: RIV-4, US-28, US-29, US-30
</commit_message>
<xml_diff>
--- a/booklets/user-stories/user-stories.xlsx
+++ b/booklets/user-stories/user-stories.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="User stories" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Screens" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User stories" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screens" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>REVIEW</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>REVIEW</t>
         </is>
       </c>
     </row>
@@ -1894,7 +1894,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>REVIEW</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(booklets): record PUC-6 status and devlog
Updates the pages table of Student_doc for the imports list and the
import detail, sets US-10, US-11 and US-12 to REVIEW, adds a dated
section to the task status log (PUC-3 and PUC-6 done) and the devlog
entry.

Refs: PUC-6, US-10, US-11, US-12
</commit_message>
<xml_diff>
--- a/booklets/user-stories/user-stories.xlsx
+++ b/booklets/user-stories/user-stories.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User stories" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screens" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="User stories" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Screens" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -954,7 +954,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>REVIEW</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>REVIEW</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>REVIEW</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(booklets): add US-38 visual revamp story and PUC-13 task
Records the visual revamp as user story US-38 (input.txt, Student_doc,
USER_STORIES and the spreadsheet) and task PUC-13 in TASKS.md.

Refs: PUC-13, US-38
</commit_message>
<xml_diff>
--- a/booklets/user-stories/user-stories.xlsx
+++ b/booklets/user-stories/user-stories.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2224,6 +2224,53 @@
       <c r="I38" s="2" t="inlineStr">
         <is>
           <t>REVIEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>US-38</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>a modern and consistent interface where the key figures stand out</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>I can read the data at a glance</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Puccetti</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Same design tokens in light and dark mode; text contrast WCAG AA in both; one brand color for highlights only, never for data (enterprise colors stay the only data colors); pill navigation usable by keyboard with the current page announced; layout usable from 375 px wide; no new dependency (system font)</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>TODO</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(booklets): add US-39 road distances story and PUC-14 task
US-39: the planner uses real road distances and driving times from an
optional self-hosted OSRM, falling back to the straight-line estimate.
PUC-14 records the task; it touches the planning engine and planner
page, so Marzella reviews it.

Refs: PUC-14, US-39
</commit_message>
<xml_diff>
--- a/booklets/user-stories/user-stories.xlsx
+++ b/booklets/user-stories/user-stories.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2271,6 +2271,53 @@
       <c r="I39" s="2" t="inlineStr">
         <is>
           <t>TODO</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>US-39</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Analyst</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>the planner to use real road distances and driving times</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>every planned day can really be driven within the working hours</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>S8</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Puccetti</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Optional self-hosted OSRM (Docker Compose profile with the OpenStreetMap extract of central Italy), so customer coordinates never leave the system; one distance and time table per import and base, about 1 s for 1,000 points and kept in memory; when the road network is off or unreachable the plan uses the straight-line estimate and says which one it used</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
         </is>
       </c>
     </row>

</xml_diff>